<commit_message>
Swing: permanent CSV record of every scan; workbook rebuilt from it
swing_store.py writes each scan once, in full, under history/swing/:
runs.csv (backdrop, NIFTY 500 close, code commit, the exact swing settings),
scans/YYYY-MM.csv (every eligible stock with score components, plan and raw
inputs) and members.csv (the universe, when it changes: a point-in-time
universe). Append-only; --force replaces one scan. Outcomes are not stored:
they are replayed from prices with each scan's own plan.

record_swing.py now writes to that record and rebuilds swing_picks.xlsx
from it, so the workbook is a report rather than the store. The 13-Oct
Nifty 200 scan is migrated (same picks), plus the 13-Oct Nifty 500 scan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/history/swing_picks.xlsx
+++ b/history/swing_picks.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -940,7 +940,7 @@
         <v>4869</v>
       </c>
       <c r="L6" t="n">
-        <v>4879.87</v>
+        <v>4879.88</v>
       </c>
       <c r="M6" t="n">
         <v>4560.6</v>
@@ -1362,6 +1362,786 @@
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F12" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>SANSERA</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4254.8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>4268.26</v>
+      </c>
+      <c r="M12" t="n">
+        <v>3953.37</v>
+      </c>
+      <c r="N12" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4740.6</v>
+      </c>
+      <c r="P12" t="n">
+        <v>5212.94</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Automobile and Auto Components</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F13" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>KALYANKJIL</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="K13" t="n">
+        <v>571</v>
+      </c>
+      <c r="L13" t="n">
+        <v>572.5700000000001</v>
+      </c>
+      <c r="M13" t="n">
+        <v>537.42</v>
+      </c>
+      <c r="N13" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="O13" t="n">
+        <v>625.3099999999999</v>
+      </c>
+      <c r="P13" t="n">
+        <v>678.04</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Consumer Durables</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F14" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PAYTM</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1715</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1716.71</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1540.76</v>
+      </c>
+      <c r="N14" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1980.65</v>
+      </c>
+      <c r="P14" t="n">
+        <v>2244.58</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F15" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="K15" t="n">
+        <v>160</v>
+      </c>
+      <c r="L15" t="n">
+        <v>160.24</v>
+      </c>
+      <c r="M15" t="n">
+        <v>150.22</v>
+      </c>
+      <c r="N15" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="O15" t="n">
+        <v>175.28</v>
+      </c>
+      <c r="P15" t="n">
+        <v>190.31</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Automobile and Auto Components</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F16" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>GABRIEL</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1411.9</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1424.22</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1303.18</v>
+      </c>
+      <c r="N16" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1605.79</v>
+      </c>
+      <c r="P16" t="n">
+        <v>1787.36</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Automobile and Auto Components</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F17" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>MAHABANK</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="K17" t="n">
+        <v>83.73999999999999</v>
+      </c>
+      <c r="L17" t="n">
+        <v>84.17</v>
+      </c>
+      <c r="M17" t="n">
+        <v>79.29000000000001</v>
+      </c>
+      <c r="N17" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="O17" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="P17" t="n">
+        <v>98.81999999999999</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F18" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G18" t="n">
+        <v>7</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="K18" t="n">
+        <v>4869</v>
+      </c>
+      <c r="L18" t="n">
+        <v>4879.88</v>
+      </c>
+      <c r="M18" t="n">
+        <v>4560.6</v>
+      </c>
+      <c r="N18" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="O18" t="n">
+        <v>5358.79</v>
+      </c>
+      <c r="P18" t="n">
+        <v>5837.7</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Capital Goods</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F19" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G19" t="n">
+        <v>8</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>TEGA</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1993.6</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2020.32</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1841.42</v>
+      </c>
+      <c r="N19" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="O19" t="n">
+        <v>2288.66</v>
+      </c>
+      <c r="P19" t="n">
+        <v>2557.01</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Capital Goods</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F20" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G20" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>MANAPPURAM</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="K20" t="n">
+        <v>326.75</v>
+      </c>
+      <c r="L20" t="n">
+        <v>327.08</v>
+      </c>
+      <c r="M20" t="n">
+        <v>301.23</v>
+      </c>
+      <c r="N20" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="O20" t="n">
+        <v>365.85</v>
+      </c>
+      <c r="P20" t="n">
+        <v>404.63</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" s="2" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nifty500</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>unfavourable</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F21" t="n">
+        <v>22090</v>
+      </c>
+      <c r="G21" t="n">
+        <v>10</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>KAJARIACER</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>pullback</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1226.7</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1236.64</v>
+      </c>
+      <c r="M21" t="n">
+        <v>1192.66</v>
+      </c>
+      <c r="N21" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1302.59</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1368.55</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Consumer Durables</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" s="2" t="n">
         <v>46308</v>
       </c>
     </row>
@@ -1402,7 +2182,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -1412,7 +2192,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">

</xml_diff>